<commit_message>
Updated UZB_grids_kan15 model - 2026-10-13 19:00
</commit_message>
<xml_diff>
--- a/VerveStacks_UZB_grids_kan15/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_UZB_grids_kan15/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_UZB_grids_kan15\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682583D4-1A00-435B-8E57-91B83FD78EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD05CC7B-4C31-407F-8173-ECDD498FDD0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="1" r:id="rId1"/>
@@ -2473,27 +2473,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:R13"/>
-  <sheetFormatPr defaultColWidth="14.73046875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.59765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.19921875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.06640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.33203125" customWidth="1"/>
-    <col min="23" max="23" width="2.73046875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.28515625" customWidth="1"/>
+    <col min="23" max="23" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:18">
@@ -2857,9 +2857,9 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BE5615C-48EE-486D-BBB8-587273C2EF02}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F952651-D613-4E1A-BC66-E74E59ED9935}">
   <dimension ref="B9:L74"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="9" spans="2:12">
       <c r="B9" t="s">
@@ -4765,14 +4765,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G82"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.06640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.46484375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.53125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.25" customHeight="1" thickBot="1">
@@ -5781,16 +5781,16 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -5833,9 +5833,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:H579"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -20796,14 +20796,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr codeName="Sheet31"/>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
@@ -20923,30 +20923,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A1:U43"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="16.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.86328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.59765625" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="8.73046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.1328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4.53125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.59765625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.53125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="2.1328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.86328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.3984375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="107.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="2.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="107.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="17.25" customHeight="1" thickBot="1">
@@ -21790,16 +21790,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="C1:L4"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="4" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.06640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.73046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.73046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -21897,9 +21895,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A3:S23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="19" width="19.265625" customWidth="1"/>
+    <col min="1" max="19" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:19" ht="17.25" customHeight="1" thickBot="1">
@@ -22257,10 +22255,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22503,7 +22501,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
   </cols>
@@ -22638,11 +22636,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22769,11 +22767,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C32"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -23106,9 +23104,9 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F641A7C3-F449-41C9-B01F-B090115F1012}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1D3C488-B75C-4184-B0C2-632F5B2F4A8B}">
   <dimension ref="B9:H74"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="9" spans="2:8">
       <c r="B9" t="s">

</xml_diff>